<commit_message>
Refactor assessment and course models to limit total_score, credits
Add new models for core file import assignment scores upload and retrieval, including 200, 400, and 404 responses.

Update core file import assignment scores upload body to require a file and add resolution_policy.

Enhance API model index to include new core file import assignment scores types.

Update V1 models for core file import assignment scores upload and retrieval with similar changes.

Modify Vite configuration to enable CSS minification with esbuild.
</commit_message>
<xml_diff>
--- a/docs/data/sample3.xlsx
+++ b/docs/data/sample3.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\erenimo\projects\ses\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\erenimo\projects\ses\docs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF7E42D-07E2-46F1-A169-CC4CF0F811C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D56AAB-5ECB-4A55-B795-72F96EAE443D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -284,9 +284,6 @@
     <t>Project(%10)_0833AB</t>
   </si>
   <si>
-    <t>221400026</t>
-  </si>
-  <si>
     <t>221400027</t>
   </si>
   <si>
@@ -354,6 +351,9 @@
   </si>
   <si>
     <t>221400049</t>
+  </si>
+  <si>
+    <t>221400025</t>
   </si>
 </sst>
 </file>
@@ -1707,7 +1707,7 @@
         <v>7</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>34</v>
@@ -1722,20 +1722,19 @@
         <v>7</v>
       </c>
       <c r="G2" s="9">
-        <f t="shared" ref="G2:H26" ca="1" si="0">TRUNC(60 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="H2" s="9">
         <f ca="1">TRUNC(60 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="I2" s="9">
         <f ca="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="J2" s="9">
         <f ca="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="K2" s="6"/>
     </row>
@@ -1744,7 +1743,7 @@
         <v>9</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>35</v>
@@ -1759,20 +1758,19 @@
         <v>7</v>
       </c>
       <c r="G3" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>80</v>
+        <v>125</v>
       </c>
       <c r="H3" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>81</v>
+        <f t="shared" ref="G3:H25" ca="1" si="0">TRUNC(60 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
+        <v>77</v>
       </c>
       <c r="I3" s="9">
-        <f t="shared" ref="I3:J26" ca="1" si="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
-        <v>44</v>
+        <f t="shared" ref="I3:J25" ca="1" si="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
+        <v>34</v>
       </c>
       <c r="J3" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="K3" s="8"/>
     </row>
@@ -1781,7 +1779,7 @@
         <v>10</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>36</v>
@@ -1797,19 +1795,19 @@
       </c>
       <c r="G4" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H4" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="I4" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="J4" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="K4" s="8"/>
     </row>
@@ -1818,7 +1816,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>37</v>
@@ -1834,19 +1832,19 @@
       </c>
       <c r="G5" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>98</v>
+        <v>65</v>
       </c>
       <c r="H5" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="I5" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J5" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="K5" s="8"/>
     </row>
@@ -1855,7 +1853,7 @@
         <v>11</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>38</v>
@@ -1875,15 +1873,15 @@
       </c>
       <c r="H6" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="I6" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="J6" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="K6" s="8"/>
     </row>
@@ -1892,7 +1890,7 @@
         <v>12</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>39</v>
@@ -1908,19 +1906,19 @@
       </c>
       <c r="G7" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="H7" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="I7" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="J7" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K7" s="8"/>
     </row>
@@ -1929,7 +1927,7 @@
         <v>13</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>40</v>
@@ -1945,19 +1943,19 @@
       </c>
       <c r="G8" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="H8" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="I8" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="J8" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="K8" s="8"/>
     </row>
@@ -1966,7 +1964,7 @@
         <v>14</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>41</v>
@@ -1982,19 +1980,19 @@
       </c>
       <c r="G9" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="H9" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>71</v>
+        <v>93</v>
       </c>
       <c r="I9" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="J9" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="K9" s="8"/>
     </row>
@@ -2003,7 +2001,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>42</v>
@@ -2019,19 +2017,19 @@
       </c>
       <c r="G10" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H10" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="I10" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J10" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K10" s="8"/>
     </row>
@@ -2040,7 +2038,7 @@
         <v>16</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>43</v>
@@ -2056,19 +2054,19 @@
       </c>
       <c r="G11" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="H11" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="I11" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="J11" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="K11" s="8"/>
     </row>
@@ -2077,7 +2075,7 @@
         <v>17</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>44</v>
@@ -2093,19 +2091,19 @@
       </c>
       <c r="G12" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="H12" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="I12" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="J12" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="K12" s="8"/>
     </row>
@@ -2114,7 +2112,7 @@
         <v>18</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>45</v>
@@ -2130,19 +2128,19 @@
       </c>
       <c r="G13" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="H13" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="I13" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="J13" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="K13" s="8"/>
     </row>
@@ -2151,7 +2149,7 @@
         <v>19</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>46</v>
@@ -2167,19 +2165,19 @@
       </c>
       <c r="G14" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="H14" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I14" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="J14" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="K14" s="8"/>
     </row>
@@ -2188,7 +2186,7 @@
         <v>20</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>47</v>
@@ -2204,11 +2202,11 @@
       </c>
       <c r="G15" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="H15" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="I15" s="9">
         <f t="shared" ca="1" si="1"/>
@@ -2216,7 +2214,7 @@
       </c>
       <c r="J15" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="K15" s="8"/>
     </row>
@@ -2225,7 +2223,7 @@
         <v>21</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>48</v>
@@ -2241,19 +2239,19 @@
       </c>
       <c r="G16" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="H16" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="I16" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J16" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="K16" s="8"/>
     </row>
@@ -2262,7 +2260,7 @@
         <v>22</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>49</v>
@@ -2278,19 +2276,19 @@
       </c>
       <c r="G17" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H17" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="I17" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="J17" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="K17" s="8"/>
     </row>
@@ -2299,7 +2297,7 @@
         <v>23</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>50</v>
@@ -2315,19 +2313,19 @@
       </c>
       <c r="G18" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="H18" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="I18" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="J18" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="K18" s="8"/>
     </row>
@@ -2336,7 +2334,7 @@
         <v>24</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>51</v>
@@ -2352,19 +2350,19 @@
       </c>
       <c r="G19" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="H19" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <v>68</v>
       </c>
       <c r="I19" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="J19" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="K19" s="8"/>
     </row>
@@ -2373,7 +2371,7 @@
         <v>25</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>52</v>
@@ -2389,19 +2387,19 @@
       </c>
       <c r="G20" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="H20" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="I20" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="J20" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="K20" s="8"/>
     </row>
@@ -2410,7 +2408,7 @@
         <v>26</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>53</v>
@@ -2426,19 +2424,19 @@
       </c>
       <c r="G21" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="H21" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="I21" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="J21" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="K21" s="8"/>
     </row>
@@ -2447,7 +2445,7 @@
         <v>27</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>54</v>
@@ -2463,19 +2461,19 @@
       </c>
       <c r="G22" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="H22" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>66</v>
+        <v>93</v>
       </c>
       <c r="I22" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="J22" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K22" s="8"/>
     </row>
@@ -2484,7 +2482,7 @@
         <v>28</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>55</v>
@@ -2500,19 +2498,19 @@
       </c>
       <c r="G23" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="H23" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I23" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J23" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K23" s="8"/>
     </row>
@@ -2521,7 +2519,7 @@
         <v>29</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>56</v>
@@ -2537,11 +2535,11 @@
       </c>
       <c r="G24" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="H24" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="I24" s="9">
         <f t="shared" ca="1" si="1"/>
@@ -2549,7 +2547,7 @@
       </c>
       <c r="J24" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="K24" s="8"/>
     </row>
@@ -2558,7 +2556,7 @@
         <v>30</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>57</v>
@@ -2574,19 +2572,19 @@
       </c>
       <c r="G25" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>98</v>
+        <v>65</v>
       </c>
       <c r="H25" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="I25" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="J25" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="K25" s="8"/>
     </row>

</xml_diff>